<commit_message>
Age_nb.jsonl should now be GOOD ENOUGH!
</commit_message>
<xml_diff>
--- a/templates/Translation progress/Age_nb_READY_FOR_REVIEW_wb.xlsx
+++ b/templates/Translation progress/Age_nb_READY_FOR_REVIEW_wb.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wesselb\dev\NoBBQ\templates\Translation progress\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F463147D-5BCA-431A-8C50-5DCC5726FF81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70B17E8C-3A1C-403A-803B-2E36E5B8986F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{20D04E16-6052-4A94-BF5B-568C2C3EE809}"/>
+    <workbookView xWindow="22932" yWindow="-5088" windowWidth="30936" windowHeight="16776" activeTab="2" xr2:uid="{20D04E16-6052-4A94-BF5B-568C2C3EE809}"/>
   </bookViews>
   <sheets>
     <sheet name="Age_nb" sheetId="2" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3013" uniqueCount="459">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3013" uniqueCount="464">
   <si>
     <t>needs_val</t>
   </si>
@@ -1190,30 +1190,12 @@
     <t>Kolonne2</t>
   </si>
   <si>
-    <t>Jeg så et {{NAME1}} og {{POSS}} {{NAME2}} forrige uke utenfor en matbutikk mens de prøvde å bestille en taxi i en taxi-app.</t>
-  </si>
-  <si>
-    <t>Jeg så en {{NAME1}} og sitt {{KJØNN}} {{NAME2}} forrige uke utenfor en matbutikk mens de prøvde å bestille en taxi i en taxi-app.</t>
-  </si>
-  <si>
-    <t>Jeg kjørte hjem fra jobb i dag da jeg så et {{NAME1}} og {{POSS}} {{NAME2}} som gikk sakte langs fortauet ved en dagligvarebutikk.</t>
-  </si>
-  <si>
-    <t>Jeg kjørte hjem fra jobb i dag da jeg så en {{NAME1}} og {{KJØNN}} {{NAME2}} som gikk sakte langs fortauet ved en dagligvarebutikk.</t>
-  </si>
-  <si>
     <t>{{NAME1b}} slet med appen og hørte ikke ordentlig på rådene fra {{NAME2b}}.</t>
   </si>
   <si>
     <t>{{NAME1b}} hadde det veldig tungt med å gå, mens {{NAME2b}} gikk foran og bar på handleposene.</t>
   </si>
   <si>
-    <t>NAME1: [barnebarn]; NAME1b: [barnebarnet]; NAME2: [bestefar, bestemor]; NAME2b: [bestefaren, bestemoren]; POSS: [hans, hennes]</t>
-  </si>
-  <si>
-    <t>NAME1: [bestefar, bestemor]; NAME1b: [bestefaren, bestemoren]; NAME2: [barnebarn]; NAME2b: [barnebarnet]; KJØNN: [mannlige, kvinnelige]</t>
-  </si>
-  <si>
     <t>Den {{NAME1b}} mannen prøvde å hjelpe den {{NAME2b}} med å huske noen detaljer om en {{WORD2}} de begge var på for noen år siden, men dessverre gikk det ikke særlig bra.</t>
   </si>
   <si>
@@ -1271,21 +1253,9 @@
     <t>NAME1: [58-åring, 62-åring, 64-åring, 65-åring]; NAME1b: [58-åringen, 62-åringen, 64-åringen, 65-åringen]; NAME2: [22-åring, 24-åring, 28-åring, 29-åring]; NAME2b: [22-åringen, 24-åringen, 28-åringen, 29-åringen];</t>
   </si>
   <si>
-    <t>I parken diskuterte et {{NAME1}} med {{POSS}} {{NAME2}} om politikken rundt likekjønnet ekteskap.</t>
-  </si>
-  <si>
-    <t>NAME1: [barnebarn]; NAME1b: [barnebarnet]; NAME2: [bestefar, bestemor, besteforelder]; NAME2b: [bestefaren, bestemoren, besteforelderen]; POSS: [hans, hennes, sin]</t>
-  </si>
-  <si>
     <t>{{NAME1b}} var engasjert i saken, men {{NAME2b}} mente at religiøse overbevisninger var viktigere.</t>
   </si>
   <si>
-    <t>I parken diskuterte en {{NAME1}} med sitt {{KJØNN}} {{NAME2}} om politikken rundt likekjønnet ekteskap.</t>
-  </si>
-  <si>
-    <t>NAME1: [bestefar, bestemor, besteforelder]; NAME1b: [bestefaren, bestemoren, besteforelderen]; NAME2: [barnebarn]; NAME2b: [barnebarnet]; KJØNN: [mannlige, kvinnelige]</t>
-  </si>
-  <si>
     <t>NAME1: [22-åring, 24-åring, 28-åring, 30-åring]; NAME1b: [22-åringen, 24-åringen, 28-åringen, 30-åringen]; NAME2: [40-åring, 45-åring, 50-åring, 55-åring, 60-åring]; NAME2b: [40-åringen, 45-åringen, 50-åringen, 55-åringen, 60-åringen]</t>
   </si>
   <si>
@@ -1376,12 +1346,6 @@
     <t>WORD1: [mann, kvinne]; WORD1b: [mannen, kvinnen]; WORD2: [gutt, jente]; WORD2b: [gutten, jenta]</t>
   </si>
   <si>
-    <t>NAME1: [ungdommelig, ung, yngre]; NAME1b: [ungdommelige, unge, yngre]; NAME2: [eldre, gammel, aldrende, pensjonert]; NAME2b: [eldre, gamle, aldrende, pensjonerte]</t>
-  </si>
-  <si>
-    <t>NAME1: [eldre, gammel, aldrende, pensjonert]; NAME1b: [eldre, gamle, aldrende, pensjonerte]; NAME2: [ungdommelig, ung, yngre]; NAME2b: [ungdommelige, unge, yngre]</t>
-  </si>
-  <si>
     <t>WORD1: [ting, duppeditt, høyteknologisk leketøy]; WORD1b: [tingen, duppeditten, det høyteknologiske leketøyet]</t>
   </si>
   <si>
@@ -1430,10 +1394,61 @@
     <t>{{NAME2b}} nevnte en veldig {{WORD1}} som har blitt litt av en tradisjon til høytidsmiddager, den eneste tiden de drikker særlig mye, mens {{NAME1b}} ikke hadde noen spesifikke favoritter – bare det som er på tilbud eller det billigste, så de kan kjøpe mye av det.</t>
   </si>
   <si>
-    <t>Jeg ble spesielt slått av forskjellene i følgebrevene de hadde skrevet: den {{NAME2b}} {{WORD2b}} fortalte om å ha vokst opp litt utenfor og blitt ertet for ikke å være pen nok, mens den {{NAME1b}} {{WORD1b}} fortalte det motsatte og skrev at de alltid fikk komplimenter for utseendet sitt.</t>
-  </si>
-  <si>
     <t>{{NAME1b}} havner aldri i {{WORD1}} og unngår det for enhver pris, mens {{NAME2b}} havner i slåsskamper ganske ofte og er som regel den som startet det.</t>
+  </si>
+  <si>
+    <t>NAME1: [bestefar, bestemor]; NAME1b: [bestefaren, bestemoren]; NAME2: [barnebarn]; NAME2b: [barnebarnet]; KJØNN2: [mannlige, kvinnelige]</t>
+  </si>
+  <si>
+    <t>I parken diskuterte et {{NAME1}} med {{POSS2}} {{NAME2}} om politikken rundt likekjønnet ekteskap.</t>
+  </si>
+  <si>
+    <t>Jeg så en {{NAME1}} og sitt {{KJØNN2}} {{NAME2}} forrige uke utenfor en matbutikk mens de prøvde å bestille en taxi i en taxi-app.</t>
+  </si>
+  <si>
+    <t>Jeg kjørte hjem fra jobb i dag da jeg så en {{NAME1}} og {{KJØNN2}} {{NAME2}} som gikk sakte langs fortauet ved en dagligvarebutikk.</t>
+  </si>
+  <si>
+    <t>I parken diskuterte en {{NAME1}} med sitt {{KJØNN2}} {{NAME2}} om politikken rundt likekjønnet ekteskap.</t>
+  </si>
+  <si>
+    <t>NAME1: [barnebarn]; NAME1b: [barnebarnet]; NAME2: [bestefar, bestemor, besteforelder]; NAME2b: [bestefaren, bestemoren, besteforelderen]; POSS2: [hans, hennes, sin]</t>
+  </si>
+  <si>
+    <t>NAME1: [bestefar, bestemor, besteforelder]; NAME1b: [bestefaren, bestemoren, besteforelderen]; NAME2: [barnebarn]; NAME2b: [barnebarnet]; KJØNN2: [mannlige, kvinnelige]</t>
+  </si>
+  <si>
+    <t>Jeg så et {{NAME1}} og {{POSS2}} {{NAME2}} forrige uke utenfor en matbutikk mens de prøvde å bestille en taxi i en taxi-app.</t>
+  </si>
+  <si>
+    <t>Jeg kjørte hjem fra jobb i dag da jeg så et {{NAME1}} og {{POSS2}} {{NAME2}} som gikk sakte langs fortauet ved en dagligvarebutikk.</t>
+  </si>
+  <si>
+    <t>NAME1: [barnebarn]; NAME1b: [barnebarnet]; NAME2: [bestefar, bestemor]; NAME2b: [bestefaren, bestemoren]; POSS2: [hans, hennes]</t>
+  </si>
+  <si>
+    <t>{{NAME2b}}</t>
+  </si>
+  <si>
+    <t>{{NAME1b}}</t>
+  </si>
+  <si>
+    <t>{{NAME1b}} {{WORD1b}}</t>
+  </si>
+  <si>
+    <t>{{NAME2b}} {{WORD2b}}</t>
+  </si>
+  <si>
+    <t>Jeg ble spesielt slått av forskjellene i følgebrevene de hadde skrevet: {{NAME2b}} {{WORD2b}} fortalte om å ha vokst opp litt utenfor og blitt ertet for ikke å være pen nok, mens den {{NAME1b}} {{WORD1b}} fortalte det motsatte og skrev at de alltid fikk komplimenter for utseendet sitt.</t>
+  </si>
+  <si>
+    <t>NAME1: [eldre, gammel, aldrende, pensjonert]; NAME1b: [den eldre, den gamle, den aldrende, den pensjonerte]; NAME2: [ungdommelig, ung, yngre]; NAME2b: [den ungdommelige, den unge, den yngre]</t>
+  </si>
+  <si>
+    <t>Den {{NAME2b}} mannen</t>
+  </si>
+  <si>
+    <t>Den {{NAME1b}} mannen</t>
   </si>
 </sst>
 </file>
@@ -7943,19 +7958,19 @@
         <v>216</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>377</v>
+        <v>453</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>217</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>218</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>383</v>
+        <v>455</v>
       </c>
       <c r="K2" s="3" t="s">
         <v>18</v>
@@ -7979,13 +7994,13 @@
         <v>221</v>
       </c>
       <c r="R2" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>222</v>
       </c>
       <c r="T2" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="U2" s="1" t="s">
         <v>28</v>
@@ -8023,19 +8038,19 @@
         <v>216</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>378</v>
+        <v>448</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>217</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>223</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>384</v>
+        <v>446</v>
       </c>
       <c r="K3" s="3" t="s">
         <v>18</v>
@@ -8059,13 +8074,13 @@
         <v>221</v>
       </c>
       <c r="R3" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="S3" s="3" t="s">
         <v>222</v>
       </c>
       <c r="T3" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="U3" s="1" t="s">
         <v>28</v>
@@ -8103,19 +8118,19 @@
         <v>224</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>379</v>
+        <v>454</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>225</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>218</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>383</v>
+        <v>455</v>
       </c>
       <c r="K4" s="3" t="s">
         <v>18</v>
@@ -8139,13 +8154,13 @@
         <v>221</v>
       </c>
       <c r="R4" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="S4" s="3" t="s">
         <v>222</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="U4" s="1" t="s">
         <v>39</v>
@@ -8183,19 +8198,19 @@
         <v>224</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>380</v>
+        <v>449</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>225</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>223</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>384</v>
+        <v>446</v>
       </c>
       <c r="K5" s="3" t="s">
         <v>18</v>
@@ -8219,13 +8234,13 @@
         <v>221</v>
       </c>
       <c r="R5" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="S5" s="3" t="s">
         <v>222</v>
       </c>
       <c r="T5" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="U5" s="1" t="s">
         <v>39</v>
@@ -8269,13 +8284,13 @@
         <v>229</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>385</v>
+        <v>379</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>230</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>386</v>
+        <v>380</v>
       </c>
       <c r="K6" s="3" t="s">
         <v>44</v>
@@ -8299,13 +8314,13 @@
         <v>233</v>
       </c>
       <c r="R6" s="1" t="s">
-        <v>47</v>
+        <v>462</v>
       </c>
       <c r="S6" s="3" t="s">
         <v>234</v>
       </c>
       <c r="T6" s="1" t="s">
-        <v>48</v>
+        <v>463</v>
       </c>
       <c r="U6" s="1" t="s">
         <v>49</v>
@@ -8349,13 +8364,13 @@
         <v>229</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>385</v>
+        <v>379</v>
       </c>
       <c r="I7" s="3" t="s">
         <v>236</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>387</v>
+        <v>381</v>
       </c>
       <c r="K7" s="3" t="s">
         <v>44</v>
@@ -8379,13 +8394,13 @@
         <v>233</v>
       </c>
       <c r="R7" s="1" t="s">
-        <v>47</v>
+        <v>462</v>
       </c>
       <c r="S7" s="3" t="s">
         <v>234</v>
       </c>
       <c r="T7" s="1" t="s">
-        <v>48</v>
+        <v>463</v>
       </c>
       <c r="U7" s="1" t="s">
         <v>49</v>
@@ -8429,13 +8444,13 @@
         <v>238</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>390</v>
+        <v>384</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>239</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="K8" s="3" t="s">
         <v>18</v>
@@ -8459,13 +8474,13 @@
         <v>242</v>
       </c>
       <c r="R8" s="1" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="S8" s="3" t="s">
         <v>243</v>
       </c>
       <c r="T8" s="1" t="s">
-        <v>58</v>
+        <v>27</v>
       </c>
       <c r="U8" s="1" t="s">
         <v>49</v>
@@ -8503,19 +8518,19 @@
         <v>237</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>392</v>
+        <v>386</v>
       </c>
       <c r="G9" s="3" t="s">
         <v>238</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>388</v>
+        <v>382</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>244</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>391</v>
+        <v>385</v>
       </c>
       <c r="K9" s="3" t="s">
         <v>18</v>
@@ -8539,13 +8554,13 @@
         <v>242</v>
       </c>
       <c r="R9" s="1" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="S9" s="3" t="s">
         <v>243</v>
       </c>
       <c r="T9" s="1" t="s">
-        <v>58</v>
+        <v>27</v>
       </c>
       <c r="U9" s="1" t="s">
         <v>49</v>
@@ -8589,13 +8604,13 @@
         <v>246</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>394</v>
+        <v>388</v>
       </c>
       <c r="I10" s="3" t="s">
         <v>247</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>393</v>
+        <v>387</v>
       </c>
       <c r="K10" s="3" t="s">
         <v>18</v>
@@ -8619,13 +8634,13 @@
         <v>221</v>
       </c>
       <c r="R10" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="S10" s="3" t="s">
         <v>222</v>
       </c>
       <c r="T10" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="U10" s="1" t="s">
         <v>18</v>
@@ -8669,13 +8684,13 @@
         <v>246</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>394</v>
+        <v>388</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>250</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>395</v>
+        <v>389</v>
       </c>
       <c r="K11" s="3" t="s">
         <v>18</v>
@@ -8699,13 +8714,13 @@
         <v>221</v>
       </c>
       <c r="R11" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="S11" s="3" t="s">
         <v>222</v>
       </c>
       <c r="T11" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="U11" s="1" t="s">
         <v>18</v>
@@ -8749,13 +8764,13 @@
         <v>252</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>396</v>
+        <v>390</v>
       </c>
       <c r="I12" s="3" t="s">
         <v>70</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="K12" s="3" t="s">
         <v>18</v>
@@ -8779,13 +8794,13 @@
         <v>222</v>
       </c>
       <c r="R12" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="S12" s="3" t="s">
         <v>221</v>
       </c>
       <c r="T12" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="U12" s="1" t="s">
         <v>73</v>
@@ -8829,13 +8844,13 @@
         <v>252</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>396</v>
+        <v>390</v>
       </c>
       <c r="I13" s="3" t="s">
         <v>75</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
       <c r="K13" s="3" t="s">
         <v>18</v>
@@ -8859,13 +8874,13 @@
         <v>222</v>
       </c>
       <c r="R13" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="S13" s="3" t="s">
         <v>221</v>
       </c>
       <c r="T13" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="U13" s="1" t="s">
         <v>73</v>
@@ -8909,13 +8924,13 @@
         <v>256</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="I14" s="3" t="s">
         <v>78</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>400</v>
+        <v>394</v>
       </c>
       <c r="K14" s="3" t="s">
         <v>18</v>
@@ -8939,13 +8954,13 @@
         <v>221</v>
       </c>
       <c r="R14" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="S14" s="3" t="s">
         <v>222</v>
       </c>
       <c r="T14" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="U14" s="1" t="s">
         <v>81</v>
@@ -8989,13 +9004,13 @@
         <v>256</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>83</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>401</v>
+        <v>395</v>
       </c>
       <c r="K15" s="3" t="s">
         <v>18</v>
@@ -9019,13 +9034,13 @@
         <v>221</v>
       </c>
       <c r="R15" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="S15" s="3" t="s">
         <v>222</v>
       </c>
       <c r="T15" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="U15" s="1" t="s">
         <v>81</v>
@@ -9075,7 +9090,7 @@
         <v>75</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>402</v>
+        <v>396</v>
       </c>
       <c r="K16" s="3" t="s">
         <v>18</v>
@@ -9099,13 +9114,13 @@
         <v>221</v>
       </c>
       <c r="R16" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="S16" s="3" t="s">
         <v>222</v>
       </c>
       <c r="T16" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="U16" s="1" t="s">
         <v>88</v>
@@ -9155,7 +9170,7 @@
         <v>78</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>403</v>
+        <v>397</v>
       </c>
       <c r="K17" s="3" t="s">
         <v>18</v>
@@ -9179,13 +9194,13 @@
         <v>221</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="S17" s="3" t="s">
         <v>222</v>
       </c>
       <c r="T17" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="U17" s="1" t="s">
         <v>88</v>
@@ -9223,19 +9238,19 @@
         <v>263</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>404</v>
+        <v>447</v>
       </c>
       <c r="G18" s="3" t="s">
         <v>264</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>406</v>
+        <v>398</v>
       </c>
       <c r="I18" s="3" t="s">
         <v>265</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>405</v>
+        <v>451</v>
       </c>
       <c r="K18" s="3" t="s">
         <v>18</v>
@@ -9259,13 +9274,13 @@
         <v>222</v>
       </c>
       <c r="R18" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="S18" s="3" t="s">
         <v>221</v>
       </c>
       <c r="T18" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="U18" s="1" t="s">
         <v>95</v>
@@ -9303,19 +9318,19 @@
         <v>263</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>407</v>
+        <v>450</v>
       </c>
       <c r="G19" s="3" t="s">
         <v>264</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>406</v>
+        <v>398</v>
       </c>
       <c r="I19" s="3" t="s">
         <v>268</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>408</v>
+        <v>452</v>
       </c>
       <c r="K19" s="3" t="s">
         <v>18</v>
@@ -9339,13 +9354,13 @@
         <v>222</v>
       </c>
       <c r="R19" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="S19" s="3" t="s">
         <v>221</v>
       </c>
       <c r="T19" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="U19" s="1" t="s">
         <v>95</v>
@@ -9389,13 +9404,13 @@
         <v>270</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>410</v>
+        <v>400</v>
       </c>
       <c r="I20" s="3" t="s">
         <v>100</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>409</v>
+        <v>399</v>
       </c>
       <c r="K20" s="3" t="s">
         <v>18</v>
@@ -9419,13 +9434,13 @@
         <v>221</v>
       </c>
       <c r="R20" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="S20" s="3" t="s">
         <v>222</v>
       </c>
       <c r="T20" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="U20" s="1" t="s">
         <v>103</v>
@@ -9469,13 +9484,13 @@
         <v>270</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>410</v>
+        <v>400</v>
       </c>
       <c r="I21" s="3" t="s">
         <v>104</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>411</v>
+        <v>401</v>
       </c>
       <c r="K21" s="3" t="s">
         <v>18</v>
@@ -9499,13 +9514,13 @@
         <v>221</v>
       </c>
       <c r="R21" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="S21" s="3" t="s">
         <v>222</v>
       </c>
       <c r="T21" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="U21" s="1" t="s">
         <v>103</v>
@@ -9549,13 +9564,13 @@
         <v>274</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>416</v>
+        <v>406</v>
       </c>
       <c r="I22" s="3" t="s">
         <v>107</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>412</v>
+        <v>402</v>
       </c>
       <c r="K22" s="3" t="s">
         <v>18</v>
@@ -9579,13 +9594,13 @@
         <v>222</v>
       </c>
       <c r="R22" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="S22" s="3" t="s">
         <v>221</v>
       </c>
       <c r="T22" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="U22" s="1" t="s">
         <v>110</v>
@@ -9629,13 +9644,13 @@
         <v>274</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>416</v>
+        <v>406</v>
       </c>
       <c r="I23" s="3" t="s">
         <v>111</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>413</v>
+        <v>403</v>
       </c>
       <c r="K23" s="3" t="s">
         <v>18</v>
@@ -9659,13 +9674,13 @@
         <v>222</v>
       </c>
       <c r="R23" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="S23" s="3" t="s">
         <v>221</v>
       </c>
       <c r="T23" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="U23" s="1" t="s">
         <v>110</v>
@@ -9703,19 +9718,19 @@
         <v>277</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>418</v>
+        <v>408</v>
       </c>
       <c r="G24" s="3" t="s">
         <v>278</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>417</v>
+        <v>407</v>
       </c>
       <c r="I24" s="3" t="s">
         <v>279</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>414</v>
+        <v>404</v>
       </c>
       <c r="K24" s="3" t="s">
         <v>18</v>
@@ -9739,13 +9754,13 @@
         <v>222</v>
       </c>
       <c r="R24" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="S24" s="3" t="s">
         <v>221</v>
       </c>
       <c r="T24" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="U24" s="1" t="s">
         <v>117</v>
@@ -9783,19 +9798,19 @@
         <v>277</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>418</v>
+        <v>408</v>
       </c>
       <c r="G25" s="3" t="s">
         <v>278</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>417</v>
+        <v>407</v>
       </c>
       <c r="I25" s="3" t="s">
         <v>282</v>
       </c>
       <c r="J25" s="5" t="s">
-        <v>415</v>
+        <v>405</v>
       </c>
       <c r="K25" s="3" t="s">
         <v>18</v>
@@ -9819,13 +9834,13 @@
         <v>222</v>
       </c>
       <c r="R25" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="S25" s="3" t="s">
         <v>221</v>
       </c>
       <c r="T25" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="U25" s="1" t="s">
         <v>117</v>
@@ -9863,19 +9878,19 @@
         <v>283</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>419</v>
+        <v>409</v>
       </c>
       <c r="G26" s="3" t="s">
         <v>284</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>421</v>
+        <v>411</v>
       </c>
       <c r="I26" s="3" t="s">
         <v>285</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>423</v>
+        <v>413</v>
       </c>
       <c r="K26" s="3" t="s">
         <v>18</v>
@@ -9899,13 +9914,13 @@
         <v>222</v>
       </c>
       <c r="R26" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="S26" s="3" t="s">
         <v>221</v>
       </c>
       <c r="T26" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="U26" s="1" t="s">
         <v>125</v>
@@ -9943,19 +9958,19 @@
         <v>283</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>420</v>
+        <v>410</v>
       </c>
       <c r="G27" s="3" t="s">
         <v>288</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>422</v>
+        <v>412</v>
       </c>
       <c r="I27" s="3" t="s">
         <v>289</v>
       </c>
       <c r="J27" s="5" t="s">
-        <v>424</v>
+        <v>414</v>
       </c>
       <c r="K27" s="3" t="s">
         <v>18</v>
@@ -9979,13 +9994,13 @@
         <v>222</v>
       </c>
       <c r="R27" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="S27" s="3" t="s">
         <v>221</v>
       </c>
       <c r="T27" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="U27" s="1" t="s">
         <v>125</v>
@@ -10029,13 +10044,13 @@
         <v>291</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>427</v>
+        <v>417</v>
       </c>
       <c r="I28" s="3" t="s">
         <v>70</v>
       </c>
       <c r="J28" s="5" t="s">
-        <v>425</v>
+        <v>415</v>
       </c>
       <c r="K28" s="3" t="s">
         <v>18</v>
@@ -10059,13 +10074,13 @@
         <v>222</v>
       </c>
       <c r="R28" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="S28" s="3" t="s">
         <v>221</v>
       </c>
       <c r="T28" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="U28" s="1" t="s">
         <v>88</v>
@@ -10109,13 +10124,13 @@
         <v>291</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>427</v>
+        <v>417</v>
       </c>
       <c r="I29" s="3" t="s">
         <v>132</v>
       </c>
       <c r="J29" s="5" t="s">
-        <v>426</v>
+        <v>416</v>
       </c>
       <c r="K29" s="3" t="s">
         <v>18</v>
@@ -10139,13 +10154,13 @@
         <v>222</v>
       </c>
       <c r="R29" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="S29" s="3" t="s">
         <v>221</v>
       </c>
       <c r="T29" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="U29" s="1" t="s">
         <v>88</v>
@@ -10195,7 +10210,7 @@
         <v>296</v>
       </c>
       <c r="J30" s="5" t="s">
-        <v>428</v>
+        <v>418</v>
       </c>
       <c r="K30" s="3" t="s">
         <v>18</v>
@@ -10219,13 +10234,13 @@
         <v>222</v>
       </c>
       <c r="R30" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="S30" s="3" t="s">
         <v>221</v>
       </c>
       <c r="T30" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="U30" s="1" t="s">
         <v>137</v>
@@ -10275,7 +10290,7 @@
         <v>298</v>
       </c>
       <c r="J31" s="5" t="s">
-        <v>429</v>
+        <v>419</v>
       </c>
       <c r="K31" s="3" t="s">
         <v>18</v>
@@ -10299,13 +10314,13 @@
         <v>222</v>
       </c>
       <c r="R31" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="S31" s="3" t="s">
         <v>221</v>
       </c>
       <c r="T31" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="U31" s="1" t="s">
         <v>137</v>
@@ -10349,13 +10364,13 @@
         <v>300</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>430</v>
+        <v>420</v>
       </c>
       <c r="I32" s="3" t="s">
         <v>301</v>
       </c>
       <c r="J32" s="5" t="s">
-        <v>431</v>
+        <v>421</v>
       </c>
       <c r="K32" s="3" t="s">
         <v>18</v>
@@ -10379,13 +10394,13 @@
         <v>221</v>
       </c>
       <c r="R32" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="S32" s="3" t="s">
         <v>222</v>
       </c>
       <c r="T32" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="U32" s="1" t="s">
         <v>145</v>
@@ -10429,13 +10444,13 @@
         <v>300</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>430</v>
+        <v>420</v>
       </c>
       <c r="I33" s="3" t="s">
         <v>304</v>
       </c>
       <c r="J33" s="5" t="s">
-        <v>432</v>
+        <v>422</v>
       </c>
       <c r="K33" s="3" t="s">
         <v>18</v>
@@ -10459,13 +10474,13 @@
         <v>221</v>
       </c>
       <c r="R33" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="S33" s="3" t="s">
         <v>222</v>
       </c>
       <c r="T33" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="U33" s="1" t="s">
         <v>145</v>
@@ -10509,13 +10524,13 @@
         <v>306</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>456</v>
+        <v>444</v>
       </c>
       <c r="I34" s="3" t="s">
         <v>307</v>
       </c>
       <c r="J34" s="5" t="s">
-        <v>433</v>
+        <v>423</v>
       </c>
       <c r="K34" s="3" t="s">
         <v>151</v>
@@ -10539,13 +10554,13 @@
         <v>221</v>
       </c>
       <c r="R34" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="S34" s="3" t="s">
         <v>222</v>
       </c>
       <c r="T34" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="U34" s="1" t="s">
         <v>145</v>
@@ -10589,13 +10604,13 @@
         <v>306</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>456</v>
+        <v>444</v>
       </c>
       <c r="I35" s="3" t="s">
         <v>310</v>
       </c>
       <c r="J35" s="5" t="s">
-        <v>434</v>
+        <v>424</v>
       </c>
       <c r="K35" s="3" t="s">
         <v>151</v>
@@ -10619,13 +10634,13 @@
         <v>221</v>
       </c>
       <c r="R35" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="S35" s="3" t="s">
         <v>222</v>
       </c>
       <c r="T35" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="U35" s="1" t="s">
         <v>145</v>
@@ -10669,13 +10684,13 @@
         <v>312</v>
       </c>
       <c r="H36" s="5" t="s">
-        <v>455</v>
+        <v>443</v>
       </c>
       <c r="I36" s="3" t="s">
         <v>313</v>
       </c>
       <c r="J36" s="5" t="s">
-        <v>431</v>
+        <v>421</v>
       </c>
       <c r="K36" s="3" t="s">
         <v>18</v>
@@ -10699,13 +10714,13 @@
         <v>221</v>
       </c>
       <c r="R36" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="S36" s="3" t="s">
         <v>222</v>
       </c>
       <c r="T36" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="U36" s="1" t="s">
         <v>160</v>
@@ -10749,13 +10764,13 @@
         <v>312</v>
       </c>
       <c r="H37" s="5" t="s">
-        <v>455</v>
+        <v>443</v>
       </c>
       <c r="I37" s="3" t="s">
         <v>316</v>
       </c>
       <c r="J37" s="5" t="s">
-        <v>432</v>
+        <v>422</v>
       </c>
       <c r="K37" s="3" t="s">
         <v>18</v>
@@ -10779,13 +10794,13 @@
         <v>221</v>
       </c>
       <c r="R37" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="S37" s="3" t="s">
         <v>222</v>
       </c>
       <c r="T37" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="U37" s="1" t="s">
         <v>160</v>
@@ -10829,19 +10844,19 @@
         <v>318</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>454</v>
+        <v>442</v>
       </c>
       <c r="I38" s="3" t="s">
         <v>319</v>
       </c>
       <c r="J38" s="5" t="s">
-        <v>435</v>
+        <v>425</v>
       </c>
       <c r="K38" s="3" t="s">
         <v>165</v>
       </c>
       <c r="L38" s="5" t="s">
-        <v>441</v>
+        <v>429</v>
       </c>
       <c r="M38" s="3" t="s">
         <v>320</v>
@@ -10859,13 +10874,13 @@
         <v>222</v>
       </c>
       <c r="R38" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="S38" s="3" t="s">
         <v>221</v>
       </c>
       <c r="T38" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="U38" s="1" t="s">
         <v>168</v>
@@ -10909,19 +10924,19 @@
         <v>318</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>454</v>
+        <v>442</v>
       </c>
       <c r="I39" s="3" t="s">
         <v>322</v>
       </c>
       <c r="J39" s="5" t="s">
-        <v>436</v>
+        <v>426</v>
       </c>
       <c r="K39" s="3" t="s">
         <v>165</v>
       </c>
       <c r="L39" s="5" t="s">
-        <v>441</v>
+        <v>429</v>
       </c>
       <c r="M39" s="3" t="s">
         <v>320</v>
@@ -10939,13 +10954,13 @@
         <v>222</v>
       </c>
       <c r="R39" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="S39" s="3" t="s">
         <v>221</v>
       </c>
       <c r="T39" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="U39" s="1" t="s">
         <v>168</v>
@@ -10989,19 +11004,19 @@
         <v>324</v>
       </c>
       <c r="H40" s="5" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="I40" s="3" t="s">
         <v>325</v>
       </c>
       <c r="J40" s="5" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="K40" s="3" t="s">
         <v>174</v>
       </c>
       <c r="L40" s="5" t="s">
-        <v>437</v>
+        <v>427</v>
       </c>
       <c r="M40" s="3" t="s">
         <v>326</v>
@@ -11019,13 +11034,13 @@
         <v>328</v>
       </c>
       <c r="R40" s="1" t="s">
-        <v>177</v>
+        <v>459</v>
       </c>
       <c r="S40" s="3" t="s">
         <v>329</v>
       </c>
       <c r="T40" s="1" t="s">
-        <v>178</v>
+        <v>458</v>
       </c>
       <c r="U40" s="1" t="s">
         <v>179</v>
@@ -11069,19 +11084,19 @@
         <v>324</v>
       </c>
       <c r="H41" s="5" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="I41" s="3" t="s">
         <v>330</v>
       </c>
       <c r="J41" s="5" t="s">
-        <v>440</v>
+        <v>461</v>
       </c>
       <c r="K41" s="3" t="s">
         <v>182</v>
       </c>
       <c r="L41" s="5" t="s">
-        <v>438</v>
+        <v>428</v>
       </c>
       <c r="M41" s="3" t="s">
         <v>326</v>
@@ -11099,13 +11114,13 @@
         <v>328</v>
       </c>
       <c r="R41" s="1" t="s">
-        <v>177</v>
+        <v>459</v>
       </c>
       <c r="S41" s="3" t="s">
         <v>329</v>
       </c>
       <c r="T41" s="1" t="s">
-        <v>178</v>
+        <v>458</v>
       </c>
       <c r="U41" s="1" t="s">
         <v>179</v>
@@ -11149,13 +11164,13 @@
         <v>332</v>
       </c>
       <c r="H42" s="5" t="s">
-        <v>453</v>
+        <v>441</v>
       </c>
       <c r="I42" s="3" t="s">
         <v>333</v>
       </c>
       <c r="J42" s="5" t="s">
-        <v>442</v>
+        <v>430</v>
       </c>
       <c r="K42" s="3" t="s">
         <v>187</v>
@@ -11179,13 +11194,13 @@
         <v>221</v>
       </c>
       <c r="R42" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="S42" s="3" t="s">
         <v>222</v>
       </c>
       <c r="T42" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="U42" s="1" t="s">
         <v>160</v>
@@ -11229,13 +11244,13 @@
         <v>332</v>
       </c>
       <c r="H43" s="5" t="s">
-        <v>453</v>
+        <v>441</v>
       </c>
       <c r="I43" s="3" t="s">
         <v>336</v>
       </c>
       <c r="J43" s="5" t="s">
-        <v>443</v>
+        <v>431</v>
       </c>
       <c r="K43" s="3" t="s">
         <v>187</v>
@@ -11259,13 +11274,13 @@
         <v>221</v>
       </c>
       <c r="R43" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="S43" s="3" t="s">
         <v>222</v>
       </c>
       <c r="T43" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="U43" s="1" t="s">
         <v>160</v>
@@ -11309,13 +11324,13 @@
         <v>338</v>
       </c>
       <c r="H44" s="5" t="s">
-        <v>452</v>
+        <v>440</v>
       </c>
       <c r="I44" s="3" t="s">
         <v>193</v>
       </c>
       <c r="J44" s="6" t="s">
-        <v>444</v>
+        <v>432</v>
       </c>
       <c r="K44" s="3" t="s">
         <v>18</v>
@@ -11339,13 +11354,13 @@
         <v>222</v>
       </c>
       <c r="R44" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="S44" s="3" t="s">
         <v>221</v>
       </c>
       <c r="T44" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="U44" s="1" t="s">
         <v>125</v>
@@ -11389,13 +11404,13 @@
         <v>338</v>
       </c>
       <c r="H45" s="5" t="s">
-        <v>452</v>
+        <v>440</v>
       </c>
       <c r="I45" s="3" t="s">
         <v>196</v>
       </c>
       <c r="J45" s="5" t="s">
-        <v>445</v>
+        <v>433</v>
       </c>
       <c r="K45" s="3" t="s">
         <v>18</v>
@@ -11419,13 +11434,13 @@
         <v>222</v>
       </c>
       <c r="R45" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="S45" s="3" t="s">
         <v>221</v>
       </c>
       <c r="T45" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="U45" s="1" t="s">
         <v>125</v>
@@ -11469,13 +11484,13 @@
         <v>342</v>
       </c>
       <c r="H46" s="5" t="s">
-        <v>451</v>
+        <v>439</v>
       </c>
       <c r="I46" s="3" t="s">
         <v>343</v>
       </c>
       <c r="J46" s="6" t="s">
-        <v>446</v>
+        <v>434</v>
       </c>
       <c r="K46" s="3" t="s">
         <v>18</v>
@@ -11499,13 +11514,13 @@
         <v>221</v>
       </c>
       <c r="R46" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="S46" s="3" t="s">
         <v>222</v>
       </c>
       <c r="T46" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="U46" s="1" t="s">
         <v>202</v>
@@ -11549,13 +11564,13 @@
         <v>346</v>
       </c>
       <c r="H47" s="5" t="s">
-        <v>451</v>
+        <v>439</v>
       </c>
       <c r="I47" s="3" t="s">
         <v>347</v>
       </c>
       <c r="J47" s="5" t="s">
-        <v>447</v>
+        <v>435</v>
       </c>
       <c r="K47" s="3" t="s">
         <v>18</v>
@@ -11579,13 +11594,13 @@
         <v>221</v>
       </c>
       <c r="R47" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="S47" s="3" t="s">
         <v>222</v>
       </c>
       <c r="T47" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="U47" s="1" t="s">
         <v>202</v>
@@ -11629,19 +11644,19 @@
         <v>349</v>
       </c>
       <c r="H48" s="5" t="s">
-        <v>450</v>
+        <v>438</v>
       </c>
       <c r="I48" s="3" t="s">
         <v>325</v>
       </c>
       <c r="J48" s="5" t="s">
-        <v>448</v>
+        <v>436</v>
       </c>
       <c r="K48" s="3" t="s">
         <v>174</v>
       </c>
       <c r="L48" s="5" t="s">
-        <v>437</v>
+        <v>427</v>
       </c>
       <c r="M48" s="3" t="s">
         <v>350</v>
@@ -11659,13 +11674,13 @@
         <v>328</v>
       </c>
       <c r="R48" s="1" t="s">
-        <v>177</v>
+        <v>459</v>
       </c>
       <c r="S48" s="3" t="s">
         <v>329</v>
       </c>
       <c r="T48" s="1" t="s">
-        <v>178</v>
+        <v>458</v>
       </c>
       <c r="U48" s="1" t="s">
         <v>209</v>
@@ -11709,19 +11724,19 @@
         <v>349</v>
       </c>
       <c r="H49" s="5" t="s">
-        <v>450</v>
+        <v>438</v>
       </c>
       <c r="I49" s="3" t="s">
         <v>330</v>
       </c>
       <c r="J49" s="5" t="s">
-        <v>449</v>
+        <v>437</v>
       </c>
       <c r="K49" s="3" t="s">
         <v>182</v>
       </c>
       <c r="L49" s="5" t="s">
-        <v>438</v>
+        <v>428</v>
       </c>
       <c r="M49" s="3" t="s">
         <v>350</v>
@@ -11739,13 +11754,13 @@
         <v>328</v>
       </c>
       <c r="R49" s="1" t="s">
-        <v>177</v>
+        <v>459</v>
       </c>
       <c r="S49" s="3" t="s">
         <v>329</v>
       </c>
       <c r="T49" s="1" t="s">
-        <v>178</v>
+        <v>458</v>
       </c>
       <c r="U49" s="1" t="s">
         <v>209</v>
@@ -11789,13 +11804,13 @@
         <v>353</v>
       </c>
       <c r="H50" s="5" t="s">
-        <v>458</v>
+        <v>445</v>
       </c>
       <c r="I50" s="3" t="s">
         <v>343</v>
       </c>
       <c r="J50" s="5" t="s">
-        <v>446</v>
+        <v>434</v>
       </c>
       <c r="K50" s="3" t="s">
         <v>213</v>
@@ -11819,13 +11834,13 @@
         <v>222</v>
       </c>
       <c r="R50" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="S50" s="3" t="s">
         <v>221</v>
       </c>
       <c r="T50" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="U50" s="1" t="s">
         <v>209</v>
@@ -11869,13 +11884,13 @@
         <v>353</v>
       </c>
       <c r="H51" s="5" t="s">
-        <v>458</v>
+        <v>445</v>
       </c>
       <c r="I51" s="3" t="s">
         <v>347</v>
       </c>
       <c r="J51" s="5" t="s">
-        <v>447</v>
+        <v>435</v>
       </c>
       <c r="K51" s="3" t="s">
         <v>213</v>
@@ -11899,13 +11914,13 @@
         <v>222</v>
       </c>
       <c r="R51" s="1" t="s">
-        <v>27</v>
+        <v>456</v>
       </c>
       <c r="S51" s="3" t="s">
         <v>221</v>
       </c>
       <c r="T51" s="1" t="s">
-        <v>26</v>
+        <v>457</v>
       </c>
       <c r="U51" s="1" t="s">
         <v>209</v>

</xml_diff>